<commit_message>
Carry knockout names through byes onto later scorecards
A bye means the other side advances without playing, so a draw containing byes already
decides several later-round places before anything is played. The scorecard script only
ever looked at round1Slots, so those cards printed blank.

It now resolves the whole bracket the way the control panel does -- byes advance, and a
recorded result advances its winner -- and prints whichever names are known on every
round's card. A side that is still undecided is left blank rather than guessed, so a
card can carry one name and one empty line.

For Men's Doubles that fills three quarterfinals outright and a fourth on one side,
where before only the single playable first-round match had names.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Savets 2026/admin/output/Knockout Scorecards.xlsx
+++ b/Savets 2026/admin/output/Knockout Scorecards.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="52">
   <si>
     <t>ROUND:</t>
   </si>
@@ -192,6 +192,27 @@
   </si>
   <si>
     <t>19:30</t>
+  </si>
+  <si>
+    <t>Bernard Stewe &amp; Lindsay October</t>
+  </si>
+  <si>
+    <t>Allan Clark &amp; Gaston Koetaan</t>
+  </si>
+  <si>
+    <t>Frans Erasmus &amp; Demos Dracoulides</t>
+  </si>
+  <si>
+    <t>Simon Dimant &amp; Jose da Silva</t>
+  </si>
+  <si>
+    <t>Ashley Wesson &amp; Terence Cable</t>
+  </si>
+  <si>
+    <t>Saaliegh Jabaar &amp; Rafiq Tofa</t>
+  </si>
+  <si>
+    <t>Zahier Isaacs &amp; David Nwafo</t>
   </si>
   <si>
     <t>20:00</t>
@@ -3740,7 +3761,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="18"/>
@@ -3756,7 +3777,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="26"/>
@@ -3932,7 +3953,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="18"/>
@@ -3948,7 +3969,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="26"/>
@@ -4124,7 +4145,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="18"/>
@@ -4316,7 +4337,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="18"/>
@@ -4332,7 +4353,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="26"/>
@@ -4447,7 +4468,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>5</v>
@@ -4639,7 +4660,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>5</v>
@@ -4817,7 +4838,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3" t="s">
@@ -5009,7 +5030,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3" t="s">
@@ -5393,7 +5414,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3" t="s">
@@ -5585,7 +5606,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3" t="s">
@@ -5814,7 +5835,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -6006,7 +6027,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -6198,7 +6219,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -6390,7 +6411,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -6582,7 +6603,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -6774,7 +6795,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -6966,7 +6987,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -7158,7 +7179,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -7542,7 +7563,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -7734,7 +7755,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -7926,7 +7947,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -8118,7 +8139,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -8310,7 +8331,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -8502,7 +8523,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>
@@ -8657,7 +8678,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3" t="s">
@@ -8694,7 +8715,7 @@
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J2" s="7"/>
     </row>

</xml_diff>